<commit_message>
fix(submissions): retire the payment-proof upload stub — replaced with ID Billing link
The PAYMENT_PENDING card button was an alert() TODO stub for the old
payment-proof upload flow, a concept removed entirely in the Coretax
payment-is-filing migration (20260723000001; /api/customer/payment-proof
deleted). The correct customer action in that state is checking the
issued ID Billing, so the button now links to /tax/billing.
Dropped the dead onUploadPayment prop chain; viewBilling i18n x3.

Found while sweeping for other alert-stub submit buttons after the
/tax/umkm bug (수정요청 25번) — no others remain.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/수정 요청 사항.xlsx
+++ b/수정 요청 사항.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G51"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="4.33203125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -479,6 +479,7 @@
     <col width="10.83203125" customWidth="1" style="5" min="8" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2"/>
     <row r="3" customFormat="1" s="2">
       <c r="A3" s="7" t="inlineStr">
@@ -1245,10 +1246,14 @@
           <t>수정</t>
         </is>
       </c>
-      <c r="F28" s="1" t="n"/>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>DB 직접 확인 결과: PT. Mono Flip Global 고객의 입력 자료가 서버에 전혀 저장돼 있지 않음(월납부·급여·원천세·부가세·결산 모두 0건). 워크큐 표시 문제가 아니라 고객 입력 화면의 저장 단계 문제로 추정 — 어느 메뉴에서 입력하셨는지 알려주시면 해당 경로의 저장 버그를 추적하겠음. 최우선 조사 대상.</t>
+          <t>[처리완료 2026-08-05] 원인: 선납법인세 화면의 제출 버튼이 저장 없이 알림만 띄우는 미완성 코드였음 — 입력 자료가 서버로 전송된 적이 없었음. 수정: 제출 시 서버 저장 + 담당 상담원 워크큐 자동 생성/배정 배선, 저장 완료 안내 표시. 배포 및 검증 완료(8/8) — PT. Mono Flip Global 계정으로 다시 입력하면 상담원 화면에 나타남. 회귀 방지 테스트를 일일 자동검증에 추가함.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(workqueue): WhatsApp-style customer request modal across all panels (요청 11·18·23)
Six duplicated plain RequestModals (PPh21 incl. bulk, 원천세, 부가세,
선납, 연신고, 직원인사) replaced with one shared RequestChatModal:
teal header with target avatar, chat-canvas body with a context pill,
the draft shown as an editable outgoing green bubble with time+✓ meta,
and a round send button. POST /request behavior unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/수정 요청 사항.xlsx
+++ b/수정 요청 사항.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/winwaysystems/mywork/ai-pajak/ai-pajak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3BD6FC-34EB-D142-82B2-7C665F9869E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99F5EE0-B537-5240-811E-6A628E7E3889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="31900" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="상담원" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="64">
   <si>
     <t>No.</t>
   </si>
@@ -53,13 +53,16 @@
     <t>삭제</t>
   </si>
   <si>
-    <t>동의. 단 이 버튼은 전체화면(사이드바 없는 레이아웃)에서 유일한 복귀 경로여서 단독 삭제하면 다른 화면으로 나갈 방법이 없어짐 — 3·4번 레이아웃 개편과 묶어서 처리하면 자연 해결.</t>
+    <t>완료</t>
+  </si>
+  <si>
+    <t>[완료 2026-08-05] 동의. 단 이 버튼은 전체화면(사이드바 없는 레이아웃)에서 유일한 복귀 경로여서 단독 삭제하면 다른 화면으로 나갈 방법이 없어짐 — 3·4번 레이아웃 개편과 묶어서 처리하면 자연 해결.</t>
   </si>
   <si>
     <t>Customer Workqueue 바로 아래에 "미검토, 수정중, 전체, 기간월" 표시는 없애줘.  아래 4번을 옮기면 중복되는 표기임</t>
   </si>
   <si>
-    <t>동의. 4번(상단 가로 배치) 진행 시 상태필터를 상단으로 옮기면서 함께 정리.</t>
+    <t>[완료 2026-08-05] 동의. 4번(상단 가로 배치) 진행 시 상태필터를 상단으로 옮기면서 함께 정리.</t>
   </si>
   <si>
     <t>사이드바</t>
@@ -71,19 +74,19 @@
     <t>수정</t>
   </si>
   <si>
-    <t>가능. 마우스 올리면 펼쳐지는 아이콘 레일 패턴 적용. 1~5번+13번을 묶어 '워크큐 레이아웃 개편' 1건으로 진행 제안.</t>
+    <t>[완료 2026-08-05] 가능. 마우스 올리면 펼쳐지는 아이콘 레일 패턴 적용. 1~5번+13번을 묶어 '워크큐 레이아웃 개편' 1건으로 진행 제안.</t>
   </si>
   <si>
     <t>사이드 메뉴의 상담원 업무함은 상단에 가로로 배치</t>
   </si>
   <si>
-    <t>가능. 세목 6개 뷰를 상단 가로 탭으로 전환. 고객 워크리스트는 좌측 유지가 탐색에 유리하나 폭 축소 동의.</t>
+    <t>[완료 2026-08-05] 가능. 세목 6개 뷰를 상단 가로 탭으로 전환. 고객 워크리스트는 좌측 유지가 탐색에 유리하나 폭 축소 동의.</t>
   </si>
   <si>
     <t>사이드 메뉴 아래쪽에 "직원 인사 기록" 메뉴도 필요 없는 메뉴임</t>
   </si>
   <si>
-    <t>메뉴만 숨기고 화면·데이터는 유지 권장 — 10번 팝업 상세에서 직원 인사정보 참조에 재사용 가치 있음. (전례: PPh4(2)도 메뉴 숨김+화면 유지)</t>
+    <t>[완료 2026-08-05] 메뉴만 숨기고 화면·데이터는 유지 권장 — 10번 팝업 상세에서 직원 인사정보 참조에 재사용 가치 있음. (전례: PPh4(2)도 메뉴 숨김+화면 유지)</t>
   </si>
   <si>
     <t>개인소득세</t>
@@ -92,34 +95,34 @@
     <t>맨위에 "view as customer sees it"은 삭제</t>
   </si>
   <si>
-    <t>동의. 간단 삭제.</t>
+    <t>[완료 2026-08-05] 동의. 간단 삭제.</t>
   </si>
   <si>
     <t>상태를 요청, 완료로 표기하지 말고 상담원 확인이 완료되면 완료, 미확인 상태면 미확인, 이슈 상황이 있으면 이슈로 표기.  급여는 개별 
 상태가 완료가 아니더라도 수퍼바이저에게 일괄 승인요청이 가능하도록 해줘</t>
   </si>
   <si>
-    <t>가능. 내부적으로 이미 3단계 판정(정상/주의/문제)이 있어 표기 매핑으로 해결. '미완료 있어도 일괄 승인요청 가능'은 정책 변경 — 요청 시 수퍼바이저 화면에 미확인·이슈 건수를 함께 표시하는 조건 권장.</t>
+    <t>[완료 2026-08-05] 가능. 내부적으로 이미 3단계 판정(정상/주의/문제)이 있어 표기 매핑으로 해결. '미완료 있어도 일괄 승인요청 가능'은 정책 변경 — 요청 시 수퍼바이저 화면에 미확인·이슈 건수를 함께 표시하는 조건 권장.</t>
   </si>
   <si>
     <t>리스트 바로 위에 있는 "AI 사전검토" 는 자동으로 실행되어서 내용이 나오게 하고, 모든 수정 작업이 끝난 후 또 실행하면 변경된 
 자료를 바탕으로 해서 다시 검토의견을 내줘</t>
   </si>
   <si>
-    <t>가능. 패널 진입 시 자동 실행 + 자료 변경이 있을 때만 재분석(변경 없으면 기존 결과 재사용) 방식 권장 — AI 호출 비용 통제 목적. 재실행 버튼은 유지.</t>
+    <t>[완료 2026-08-05] 가능. 패널 진입 시 자동 실행 + 자료 변경이 있을 때만 재분석(변경 없으면 기존 결과 재사용) 방식 권장 — AI 호출 비용 통제 목적. 재실행 버튼은 유지.</t>
   </si>
   <si>
     <t xml:space="preserve">리스트 위에 있는 "일괄요청" 버튼을 삭제하고 "승인요청"으로 변경.  승인요청을 클릭하게 되면 수퍼바이저에게 요청하는 내용을 적을 수 있게 해줘. 수퍼바이저가 승인을 완료할 경우에는 이 버튼이 사라지고 버튼 위치에 "승인완료"로 표기.  만약 승인이 되지 
 않고 수정사항이 있을 경우에는 수퍼바이저가 직접 수정할 수도 있고 (색이 다르게) 메신저로 요청사항을 전달할 수도 있음.  이 내용에 수긍하면 상담원이 다시 "일괄요청" 클릭할 수 있게 해줘 </t>
   </si>
   <si>
-    <t>동의. 기존 승인/반려 흐름을 재사용하되 ①요청 코멘트 입력 ②승인완료 배지 전환 ③수퍼바이저 직접수정 시 색상 구분(수정 전/후 값 보존 필요) 신규 개발. 규모 중간.</t>
+    <t>[완료 2026-08-05] 동의. 기존 승인/반려 흐름을 재사용하되 ①요청 코멘트 입력 ②승인완료 배지 전환 ③수퍼바이저 직접수정 시 색상 구분(수정 전/후 값 보존 필요) 신규 개발. 규모 중간.</t>
   </si>
   <si>
     <t>리스트의 한 행을 클릭하면 맨 아래 선택직원 상세보기가 나타나는데, 이걸 팝업으로 변경시켜줘.  나중에 직원이 수십 수백명이 될 수 있거든….  그리고 지금은 직원 선택이 안 되고 있어.  그래서 팝업이 된 상태에서 수정사항 입력하고 "저장 및 확인" 해줘.  이 버튼을 누르면 이 급여자의 상태는 "완료"가 되는거야.  상담원이 수정한 내용은 수퍼바이저가 볼때 다른 색상으로 보여지게 해서 상담원이 뭘 수정했는지 알게 해줘.  맨 아래에 있는 직원별 AI 분석은 그대로 유지해줘</t>
   </si>
   <si>
-    <t>동의. '직원 선택이 안 됨'은 별도 버그로 확인하겠음. 수정분 색상 표시는 변경 전/후 값 기록이 필요 — 기존 직원 변경이력 구조 재사용 가능. 수백명 대비 팝업+검색 방향 타당.</t>
+    <t>[완료 2026-08-05] 동의. '직원 선택이 안 됨'은 별도 버그로 확인하겠음. 수정분 색상 표시는 변경 전/후 값 기록이 필요 — 기존 직원 변경이력 구조 재사용 가능. 수백명 대비 팝업+검색 방향 타당.</t>
   </si>
   <si>
     <t>맨 뒤의 "요청" 버튼을 누르면 고객에게 문자가 나가는 구조인데, 왓쯔앱 UI 처럼 디자인을 적용해줘.  지금은 너무 촌스러.</t>
@@ -141,7 +144,7 @@
     <t>신규</t>
   </si>
   <si>
-    <t>로그인 자체는 공용 로그인 화면을 쓰고 있음. 워크큐 상단에 프로필/로그아웃 메뉴가 없는 것이 실제 문제 — 레이아웃 개편(3·4번)에 포함해 해결.</t>
+    <t>[완료 2026-08-05] 로그인 자체는 공용 로그인 화면을 쓰고 있음. 워크큐 상단에 프로필/로그아웃 메뉴가 없는 것이 실제 문제 — 레이아웃 개편(3·4번)에 포함해 해결.</t>
   </si>
   <si>
     <t>원천세</t>
@@ -150,22 +153,22 @@
     <t xml:space="preserve">상태를 요청, 완료로 표기하지 말고 상담원 확인이 완료되면 완료, 미확인 상태면 미확인, 이슈 상황이 있으면 이슈로 표기. </t>
   </si>
   <si>
-    <t>7번과 동일 처리(공통 컴포넌트로 6개 세목 뷰에 일괄 적용).</t>
+    <t>[완료 2026-08-05] 7번과 동일 처리(공통 컴포넌트로 6개 세목 뷰에 일괄 적용).</t>
   </si>
   <si>
     <t>리스트를 더블클릭하면 상세정보가 팝업되도록 해줘.  거기서 내용 수정하고 저장할 수 있도록.  10번 개인소득세처럼.</t>
   </si>
   <si>
-    <t>동의. 10번과 공통 팝업 컴포넌트로 개발해 모든 세목에 재사용.</t>
-  </si>
-  <si>
-    <t>8번과 동일 처리.</t>
+    <t>[완료 2026-08-05] 동의. 10번과 공통 팝업 컴포넌트로 개발해 모든 세목에 재사용.</t>
+  </si>
+  <si>
+    <t>[완료 2026-08-05] 8번과 동일 처리.</t>
   </si>
   <si>
     <t>리스트 위에 "승인요청" 버튼을 만들어줘.  승인요청을 클릭하게 되면 수퍼바이저에게 요청하는 내용을 적을 수 있게 해줘. 수퍼바이저가 승인을 완료할 경우에는 이 버튼이 사라지고 버튼 위치에 "승인완료"로 표기.  만약 승인이 되지 않고 수정사항이 있을 경우에는 수퍼바이저가 직접 수정할 수도 있고 (색이 다르게) 메신저로 요청사항을 전달할 수도 있음.  이 내용에 수긍하면 상담원이 다시 "승인요청" 클릭할 수 있게 해줘 "</t>
   </si>
   <si>
-    <t>9번과 동일 처리(공통).</t>
+    <t>[완료 2026-08-05] 9번과 동일 처리(공통).</t>
   </si>
   <si>
     <t>11번과 동일 처리.</t>
@@ -177,7 +180,7 @@
     <t xml:space="preserve">상태를 요청, 완료로 표기하지 말고 상담원 확인이 완료되면 완료, 미확인 상태면 미확인, 이슈 상황이 있으면 이슈로 표기.  중간에 부가세 요율도 표기해줘.  </t>
   </si>
   <si>
-    <t>동의. 요율 컬럼 추가(사치품 여부 반영 11%/12% 자동 표기). 상태 3값은 7번과 동일 처리.</t>
+    <t>[완료 2026-08-05] 동의. 요율 컬럼 추가(사치품 여부 반영 11%/12% 자동 표기). 상태 3값은 7번과 동일 처리.</t>
   </si>
   <si>
     <t xml:space="preserve">중간에 coretax 대조가 있는데, coretax 자료를 고객사 웹페이지에 들어가는 것으로 기획되어 있는데, 그걸 여기에서 보여줘야 해.  
@@ -185,16 +188,16 @@
 옆에 "coretax에서 부가세 자료 가져오기" 버튼을 만들어서 업로드를 시켜야 해.  이 옆에 파일 업로드된  상태가 보이게 해줘.  </t>
   </si>
   <si>
-    <t>핵심 지적. 사실 이 기능은 이미 개발돼 있음 — 고객용 부가세 화면의 'Coretax 대조'(xlsx 업로드→자동 매칭: 일치/차이/누락). 이 업로드+대조 버튼을 워크큐 부가세 패널에 노출하면 되므로 기존 기능 재사용으로 규모 작음.</t>
+    <t>[완료 2026-08-05] 핵심 지적. 사실 이 기능은 이미 개발돼 있음 — 고객용 부가세 화면의 'Coretax 대조'(xlsx 업로드→자동 매칭: 일치/차이/누락). 이 업로드+대조 버튼을 워크큐 부가세 패널에 노출하면 되므로 기존 기능 재사용으로 규모 작음.</t>
   </si>
   <si>
     <t xml:space="preserve">이슈 밑에는 맨앞에 이슈로 표기된 건에 대해서만 이슈내용을 간단히 보여준다.  </t>
   </si>
   <si>
-    <t>동의. 이슈로 판정된 행만 요약 표시하도록 필터링. 간단.</t>
-  </si>
-  <si>
-    <t>15번과 동일 처리(공통 팝업).</t>
+    <t>[완료 2026-08-05] 동의. 이슈로 판정된 행만 요약 표시하도록 필터링. 간단.</t>
+  </si>
+  <si>
+    <t>[완료 2026-08-05] 15번과 동일 처리(공통 팝업).</t>
   </si>
   <si>
     <t>선납법인세</t>
@@ -205,9 +208,6 @@
 상담원에게 전달되지 않는 문제가 있어</t>
   </si>
   <si>
-    <t>완료</t>
-  </si>
-  <si>
     <t>[처리완료 2026-08-05] 원인: 선납법인세 화면의 제출 버튼이 저장 없이 알림만 띄우는 미완성 코드였음 — 입력 자료가 서버로 전송된 적이 없었음. 수정: 제출 시 서버 저장 + 담당 상담원 워크큐 자동 생성/배정 배선, 저장 완료 안내 표시. 배포 및 검증 완료(8/8) — PT. Mono Flip Global 계정으로 다시 입력하면 상담원 화면에 나타남. 회귀 방지 테스트를 일일 자동검증에 추가함.</t>
   </si>
   <si>
@@ -220,9 +220,6 @@
   </si>
   <si>
     <t>메뉴 링크는 존재(발행 보드로 연결) — '작동 안 됨' 증상 확인 필요(클릭 무반응인지, 빈 화면인지). '승인 없이 발행'은 현재 오발행 방지를 위해 승인완료 건만 발행되도록 서버가 강제 중 — 예외 발행 경로를 만들되 사유 입력+감사기록+수퍼바이저 자동통지를 조건으로 하는 방식 권장.</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>수</t>
@@ -241,7 +238,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -251,6 +248,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -282,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -306,6 +309,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -630,10 +636,10 @@
     <col min="3" max="3" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="117.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="24.6640625" style="5" customWidth="1"/>
     <col min="7" max="7" width="255.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="5" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="5"/>
+    <col min="8" max="9" width="10.83203125" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -675,9 +681,11 @@
       <c r="E4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G4" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -691,14 +699,16 @@
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G5" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -709,17 +719,19 @@
         <v>46239</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G6" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -730,17 +742,19 @@
         <v>46239</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G7" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -751,17 +765,19 @@
         <v>46239</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G8" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -772,17 +788,19 @@
         <v>46239</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G9" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -793,17 +811,19 @@
         <v>46239</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="4"/>
+      <c r="F10" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G10" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -814,17 +834,19 @@
         <v>46239</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G11" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -835,17 +857,19 @@
         <v>46239</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G12" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="96" customHeight="1" x14ac:dyDescent="0.2">
@@ -856,17 +880,19 @@
         <v>46239</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G13" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -877,17 +903,17 @@
         <v>46239</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" s="4"/>
-      <c r="G14" s="4" t="s">
-        <v>33</v>
+      <c r="G14" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="86" customHeight="1" x14ac:dyDescent="0.2">
@@ -901,14 +927,14 @@
         <v>6</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" s="4"/>
-      <c r="G15" s="4" t="s">
-        <v>35</v>
+      <c r="G15" s="9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -922,14 +948,16 @@
         <v>6</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="4"/>
+        <v>38</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G16" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -940,17 +968,19 @@
         <v>46239</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G17" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -961,17 +991,19 @@
         <v>46239</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" s="4"/>
+        <v>38</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G18" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -982,17 +1014,19 @@
         <v>46239</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G19" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -1003,17 +1037,19 @@
         <v>46239</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" s="4"/>
+        <v>38</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G20" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
@@ -1024,17 +1060,17 @@
         <v>46239</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F21" s="4"/>
-      <c r="G21" s="4" t="s">
-        <v>47</v>
+      <c r="G21" s="9" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -1045,17 +1081,19 @@
         <v>46239</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G22" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -1066,17 +1104,19 @@
         <v>46239</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G23" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="62" customHeight="1" x14ac:dyDescent="0.2">
@@ -1087,17 +1127,19 @@
         <v>46239</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="4"/>
+        <v>38</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G24" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1108,17 +1150,19 @@
         <v>46239</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G25" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1129,17 +1173,17 @@
         <v>46239</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="4"/>
+      <c r="G26" s="9" t="s">
         <v>48</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1150,17 +1194,19 @@
         <v>46239</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F27" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G27" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="68" customHeight="1" x14ac:dyDescent="0.2">
@@ -1171,16 +1217,16 @@
         <v>46239</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>59</v>
@@ -1200,10 +1246,10 @@
         <v>61</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F29" s="4"/>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="9" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1211,9 +1257,7 @@
       <c r="A30" s="1">
         <v>27</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B30" s="3"/>
       <c r="C30" s="1"/>
       <c r="D30" s="4"/>
       <c r="E30" s="1"/>
@@ -1224,9 +1268,7 @@
       <c r="A31" s="1">
         <v>28</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="B31" s="3"/>
       <c r="C31" s="1"/>
       <c r="D31" s="4"/>
       <c r="E31" s="1"/>
@@ -1239,9 +1281,7 @@
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
-      <c r="D32" s="4" t="s">
-        <v>63</v>
-      </c>
+      <c r="D32" s="4"/>
       <c r="E32" s="1"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -1447,7 +1487,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(inbox): workqueue-integrated customer inbox + per-customer internal directive history (요청 12)
- workqueue: floating '메신저/요청함' drawer (RequestDrawer) removed —
  고객 인박스 is now a sidebar menu entry alongside ID Billing 발행
- customer-inbox right pane: static customer-info/metadata cards replaced
  with the counselor↔supervisor directive history for the SELECTED
  customer — reuses operator_message INTERNAL channel (no new tables);
  supervisor notes render orange, counselor replies violet; assigned-
  operator visibility rules apply as-is
- input requires a selected customer thread, so non-customer chatter
  can't happen here (개인 메신저 몫) — per the request's policy
- SPT Masa quick-create + resolve actions preserved

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/수정 요청 사항.xlsx
+++ b/수정 요청 사항.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/winwaysystems/mywork/ai-pajak/ai-pajak/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99F5EE0-B537-5240-811E-6A628E7E3889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92FC889-D0B7-C541-99D3-12E786EF885D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="64">
   <si>
     <t>No.</t>
   </si>
@@ -128,14 +128,14 @@
     <t>맨 뒤의 "요청" 버튼을 누르면 고객에게 문자가 나가는 구조인데, 왓쯔앱 UI 처럼 디자인을 적용해줘.  지금은 너무 촌스러.</t>
   </si>
   <si>
-    <t>동의. 고객 채팅에 이미 적용한 WhatsApp 스타일(말풍선·날짜 구분선·읽음 ✓✓)을 요청 모달에도 확장 적용.</t>
+    <t>[완료 2026-08-06] 동의. 고객 채팅에 이미 적용한 WhatsApp 스타일(말풍선·날짜 구분선·읽음 ✓✓)을 요청 모달에도 확장 적용.</t>
   </si>
   <si>
     <t>아래 메신저/요청함 버튼이 있는데, "고객 인박스 열기" 버튼을 누르면 예전에 만들어 놓은  싸이트로 연결돼.  이 버튼은 아예 삭제해줘. 
 그리고 고객 인박스를 사이드 메뉴로 옮기고 내용은 전에 만들어 놓은 화면 그대로 사용해도 돼.  단, 맨 오른쪽에 "customer info" 부분이 있는데 여기에는 상담원과 수퍼바이저의 상담내용이 나오게 해줘.  즉, 수퍼바이저가 고객이 선택된 가운데 일괄요청에 대한 의견이라던지 이 고객에 대한 내용을 상담원에게 지시하는 것은 이 창에서 이력으로 보여지게 해줘.  그러므로 수퍼바이저와 상담원은 고객과 관련되지 않은 내용이나 통상적인 내용은 메신저로 소통할 수 없어.  그런건 개인 메신저 사용하면 됨</t>
   </si>
   <si>
-    <t>가능하나 규모 큼. 인박스 화면 이식은 단순하지만 우측 customer info를 '수퍼바이저↔상담원의 고객별 지시 이력'으로 바꾸는 건 고객별 내부 대화 스레드 신설이 필요. 별도 트랙으로 분리 권장. '고객 무관 대화 차단'은 이 창에서 고객 컨텍스트 없이는 입력 불가로 처리.</t>
+    <t>가능하나 규모 큼. 인박스 화면 이식은 단순하지만 우측 customer info를 '수퍼바이저↔상담원의 고객별 지시 이력'으로 바꾸는 건 고객별 내부 대화 스레드 신설이 필요. 별도 트랙으로 분리 권장. '고객 무관 대화 차단'은 이 창에서 고객 컨텍스트 없이는 입력 불가로 처리. [다음 세션 착수 예정]</t>
   </si>
   <si>
     <t>상담원 로그인 로그아웃 화면이 없음</t>
@@ -171,7 +171,7 @@
     <t>[완료 2026-08-05] 9번과 동일 처리(공통).</t>
   </si>
   <si>
-    <t>11번과 동일 처리.</t>
+    <t>[완료 2026-08-06] 11번과 동일 처리.</t>
   </si>
   <si>
     <t>부가세</t>
@@ -238,7 +238,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -254,6 +254,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -285,7 +291,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -312,6 +318,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -638,8 +647,8 @@
     <col min="5" max="5" width="14.83203125" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.6640625" style="5" customWidth="1"/>
     <col min="7" max="7" width="255.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.83203125" style="5" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="5"/>
+    <col min="8" max="10" width="10.83203125" style="5" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="5"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -911,7 +920,9 @@
       <c r="E14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="4"/>
+      <c r="F14" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G14" s="9" t="s">
         <v>34</v>
       </c>
@@ -932,7 +943,7 @@
       <c r="E15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="4"/>
+      <c r="F15" s="10"/>
       <c r="G15" s="9" t="s">
         <v>36</v>
       </c>
@@ -1068,7 +1079,9 @@
       <c r="E21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="4"/>
+      <c r="F21" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G21" s="9" t="s">
         <v>48</v>
       </c>
@@ -1181,7 +1194,9 @@
       <c r="E26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F26" s="4"/>
+      <c r="F26" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="G26" s="9" t="s">
         <v>48</v>
       </c>
@@ -1248,7 +1263,7 @@
       <c r="E29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F29" s="4"/>
+      <c r="F29" s="10"/>
       <c r="G29" s="9" t="s">
         <v>62</v>
       </c>

</xml_diff>